<commit_message>
Feature: Adiciona métodos para o calculo da minimização e refatora os dados de entrada e saida
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,188 +413,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Order</t>
+          <t>Ordem</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Padrão</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Layout</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Layers</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Camadas</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Comprimento (m)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Aproveitamento (%)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>GG</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Total Length (m)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Cut Perimeter (m)</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Waste Area (m²)</t>
-        </is>
-      </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Cutting Cost (R$)</t>
+          <t>Custo Total</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Layout Cost (R$)</t>
+          <t>Metros Tecido</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Waste Cost (R$)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Total Cost (R$)</t>
+          <t>Desperdício (m²)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>order_1</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>No solution</t>
-        </is>
+          <t>calça</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7.921</v>
+      </c>
+      <c r="F2" t="n">
+        <v>94</v>
+      </c>
+      <c r="G2" t="n">
+        <v>24</v>
+      </c>
+      <c r="H2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" t="n">
+        <v>24</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5496.860067</v>
+      </c>
+      <c r="L2" t="n">
+        <v>279.937</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.446434</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>order_1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>calça</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7.233</v>
+      </c>
+      <c r="F3" t="n">
+        <v>91</v>
+      </c>
+      <c r="G3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H3" t="n">
+        <v>9</v>
+      </c>
+      <c r="I3" t="n">
+        <v>27</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5496.860067</v>
+      </c>
+      <c r="L3" t="n">
+        <v>279.937</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.446434</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>order_1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>calça</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
-        <v>9</v>
-      </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>80</v>
-      </c>
-      <c r="E3" t="n">
-        <v>140</v>
-      </c>
-      <c r="F3" t="n">
-        <v>60</v>
-      </c>
-      <c r="G3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.0044</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>60.37</v>
+      <c r="D4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7.001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>85</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16</v>
+      </c>
+      <c r="H4" t="n">
+        <v>32</v>
+      </c>
+      <c r="I4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J4" t="n">
+        <v>32</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5496.860067</v>
+      </c>
+      <c r="L4" t="n">
+        <v>279.937</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.446434</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Order Totals</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+          <t>order_1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>calça</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>140</v>
+        <v>7.772</v>
       </c>
       <c r="F5" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="G5" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>2.45</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>4410</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0.83</v>
+        <v>5496.860067</v>
       </c>
       <c r="L5" t="n">
-        <v>0.73</v>
+        <v>279.937</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>60.37</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>No solution</t>
-        </is>
+        <v>0.446434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>